<commit_message>
Day 1: record decisions and metrics in the build plan
Workbook: D1, D2, D5 filled with the actual seed, cohort and rationale;
D13-D15 added (A1c over glucose, CSV over FHIR, five of eighteen tables);
Metrics 1-9 plus cohort size; tasks 1.1-1.11 marked done.

LOAD_BRONZE_GUIDE.md extends the 1.12 walkthrough with the decisions to
make before writing, the traps specific to this dataset, and the lineage
column type gotcha in V1.7.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build-plan/Clinical_Care_Gap_Build_Plan.xlsx
+++ b/build-plan/Clinical_Care_Gap_Build_Plan.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day Plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQ Matrix" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Learning Log" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="START HERE" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Day Plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Task Tracker" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="DQ Matrix" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Metrics" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Learning Log" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Task Tracker'!$A$4:$H$74</definedName>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H5" s="13" t="inlineStr"/>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H6" s="13" t="inlineStr"/>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr"/>
@@ -1407,7 +1407,7 @@
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr"/>
@@ -1452,7 +1452,7 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr"/>
@@ -1488,7 +1488,7 @@
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H10" s="13" t="inlineStr"/>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr"/>
@@ -1560,10 +1560,14 @@
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H12" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="inlineStr">
+        <is>
+          <t>Row counts in Metrics 1-5. profile.py replaces the ad-hoc loop.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="62" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
@@ -1596,10 +1600,14 @@
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H13" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>8 cohort codes; 72 patients have a complication but no T2DM code. See cohort.py.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="62" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -1632,10 +1640,14 @@
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H14" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>Units are %, so DQ3 order of magnitude OK — but floor 3.0 flags 993 clean values.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="62" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
@@ -1668,10 +1680,14 @@
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H15" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>0.0% resolved → D5 decided early, no active-as-of filter needed.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="62" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -3829,7 +3845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3918,8 +3934,16 @@
           <t>Day 1</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr"/>
-      <c r="G5" s="13" t="inlineStr"/>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>1,000 (-p 1000) → 1,142 patient records</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>Synthea -p counts survivors, so 1,000 alive + 142 deceased. Keeps every query sub-second while still yielding a 161-patient cohort. Deceased are loaded but excluded from the gap denominator on Day 4.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="74" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -3947,8 +3971,16 @@
           <t>Day 1</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr"/>
-      <c r="G6" s="13" t="inlineStr"/>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Massachusetts, seed 20260823</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>The seed is the half that matters — it makes every README number reproducible by a reviewer. MA is Synthea's best-calibrated state. Note --exporter.fhir.export false alone is not enough; hospital and practitioner FHIR need their own flags.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="74" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
@@ -4034,8 +4066,16 @@
           <t>Day 4</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr"/>
-      <c r="G9" s="13" t="inlineStr"/>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Any of 8 diabetes SNOMED codes ever recorded. No active-as-of filter. Cohort = 161.</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>Decided Day 1 — the evidence arrived early. Anchoring on 44054006 alone misses 72 patients who carry a diabetic complication with no underlying dx code (45% of cohort, and the sickest half). Prediabetes 714628002 excluded: 430 patients, would triple the denominator. 0 of 819 diabetes rows have a stop date, so "ever recorded" needs no date logic. See pipeline/cohort.py.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="74" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -4239,6 +4279,117 @@
       </c>
       <c r="F16" s="13" t="inlineStr"/>
       <c r="G16" s="13" t="inlineStr"/>
+    </row>
+    <row r="17" ht="74" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Which lab defines the care gap — A1c or blood glucose</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Glucose is the larger table (9,879 vs 8,749) and covers more of the cohort. Both are reasons to reject it.</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Choosing glucose would silently break the claim that this implements a real published measure.</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>HbA1c, LOINC 4548-4. Glucose (2339-0, 2345-7) is context only, never a gap definition.</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>A1c integrates ~3 months of blood sugar; glucose is a snapshot. In our own data the within-patient, within-year spread is 6.2% of the mean for A1c vs 21.0% for glucose. Glucose is also drawn on everyone incidentally — 160 of 161 cohort patients have one vs 131 with an A1c — so its absence carries no signal. And HEDIS specifies A1c; no measure anywhere requires an annual glucose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="74" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Synthea export format — CSV or FHIR</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>FHIR JSON is more realistic interchange; CSV loads in one line of DuckDB.</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Determines how much of the seven days is spent parsing versus on the actual subject.</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>CSV (--exporter.csv.export true, all three FHIR exporters false)</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>FHIR conformance is an explicit PRD non-goal. The subject of this project is data quality, not nested resource parsing. CSV spends the time on the subject.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="74" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Which of the 18 Synthea CSVs get loaded into Bronze</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>All 18 (773 MB), or the five the care gap actually needs.</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>claims_transactions alone is 1,031,224 rows — 40% of total volume with no clinical role.</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>Five: patients, encounters, conditions, observations, medications.</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>Everything else is billing (claims, payers), or clinical data with no bearing on an A1c gap (imaging_studies, procedures, devices, supplies, allergies, careplans, immunizations). organizations/providers may be added on Day 6 if role views need facility names.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4704,7 +4855,9 @@
           <t>Bronze rows — patients</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr"/>
+      <c r="C5" s="12" t="n">
+        <v>1142</v>
+      </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
           <t>README architecture table, P2 layer counts</t>
@@ -4725,7 +4878,9 @@
           <t>Bronze rows — encounters</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr"/>
+      <c r="C6" s="12" t="n">
+        <v>65350</v>
+      </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
           <t>README architecture table, P2 layer counts</t>
@@ -4746,7 +4901,9 @@
           <t>Bronze rows — conditions</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr"/>
+      <c r="C7" s="12" t="n">
+        <v>40105</v>
+      </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
           <t>README architecture table, P2 layer counts</t>
@@ -4767,7 +4924,9 @@
           <t>Bronze rows — observations</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr"/>
+      <c r="C8" s="12" t="n">
+        <v>836111</v>
+      </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
           <t>README architecture table, P2 layer counts</t>
@@ -4788,7 +4947,9 @@
           <t>Bronze rows — medications</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr"/>
+      <c r="C9" s="12" t="n">
+        <v>56228</v>
+      </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
           <t>README architecture table, P2 layer counts</t>
@@ -4809,7 +4970,11 @@
           <t>Distinct diabetes SNOMED codes found</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr"/>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>8 in cohort (9 matched "%diabet%"; prediabetes 714628002 excluded)</t>
+        </is>
+      </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
           <t>DATA_DICTIONARY.md code table</t>
@@ -4830,7 +4995,11 @@
           <t>A1c LOINC code confirmed</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr"/>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>4548-4 — Hemoglobin A1c/Hemoglobin.total in Blood, units "%"</t>
+        </is>
+      </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
           <t>DATA_DICTIONARY.md code table</t>
@@ -4851,7 +5020,11 @@
           <t>A1c value range (min / median / max)</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr"/>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>2.3 / 5.2 / 8.8  (n=8,749; 993 below DQ3 floor of 3.0 → revise floor to 2.0)</t>
+        </is>
+      </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Sanity check for DQ3's 3.0-20.0 bounds</t>
@@ -4872,7 +5045,11 @@
           <t>% of diabetes conditions with a resolved_date</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr"/>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>0.0%  (0 of 819 diabetes condition rows have a STOP date)</t>
+        </is>
+      </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Decides cohort definition D5</t>
@@ -5019,7 +5196,9 @@
           <t>Diabetic patients in cohort (denominator)</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr"/>
+      <c r="C20" s="12" t="n">
+        <v>161</v>
+      </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
           <t>README result line, P1 headline</t>
@@ -5082,7 +5261,9 @@
           <t>Patients never tested for A1c</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr"/>
+      <c r="C23" s="12" t="n">
+        <v>30</v>
+      </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
           <t>P3 — the highest-risk subgroup</t>
@@ -5090,7 +5271,7 @@
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>Day 4</t>
+          <t>Day 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pin all four Synthea time flags after V1.3 failed; regenerate and refresh
V1.3 (regenerate with the same seed, compare) failed four weeks after the
original run: 1,151 patients instead of 1,142, every table 4-6% larger.
-s pins only the patient RNG. The clinician seed (-cs), reference date (-r)
and end date (-e) all default to the wall clock; each was found by fixing
one and seeing what still moved. With all four, two runs are identical in
content across every table.

data/raw regenerated with the pinned command, Bronze reloaded, and every
number in the docs, cohort.py and the workbook refreshed from it. Cohort is
still 161; open A1c gap is now 69 of 161.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build-plan/Clinical_Care_Gap_Build_Plan.xlsx
+++ b/build-plan/Clinical_Care_Gap_Build_Plan.xlsx
@@ -1491,7 +1491,11 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H10" s="13" t="inlineStr"/>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>V1.3 failed with -s alone (data grew 4-6% four weeks later). Fixed with -cs -r -e; regenerated 2026-09-20. Full command in DAY_1_DECISIONS.md D2.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="62" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
@@ -1605,7 +1609,7 @@
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>8 cohort codes; 72 patients have a complication but no T2DM code. See cohort.py.</t>
+          <t>8 cohort codes; 73 patients have a complication but no T2DM code. See cohort.py.</t>
         </is>
       </c>
     </row>
@@ -1645,7 +1649,7 @@
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>Units are %, so DQ3 order of magnitude OK — but floor 3.0 flags 993 clean values.</t>
+          <t>Units are %, so DQ3 order of magnitude OK — but floor 3.0 flags 951 clean values.</t>
         </is>
       </c>
     </row>
@@ -3936,12 +3940,12 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>1,000 (-p 1000) → 1,142 patient records</t>
+          <t>1,000 (-p 1000) → 1,153 patient records</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>Synthea -p counts survivors, so 1,000 alive + 142 deceased. Keeps every query sub-second while still yielding a 161-patient cohort. Deceased are loaded but excluded from the gap denominator on Day 4.</t>
+          <t>Synthea -p counts survivors, so 1,000 alive + 153 deceased. Keeps every query sub-second while still yielding a 161-patient cohort. Deceased are loaded but excluded from the gap denominator on Day 4.</t>
         </is>
       </c>
     </row>
@@ -3973,12 +3977,12 @@
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>Massachusetts, seed 20260823</t>
+          <t>Massachusetts; -s 20260823 -cs 20260823 -r 20260823 -e 20260823</t>
         </is>
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>The seed is the half that matters — it makes every README number reproducible by a reviewer. MA is Synthea's best-calibrated state. Note --exporter.fhir.export false alone is not enough; hospital and practitioner FHIR need their own flags.</t>
+          <t>V1.3 FAILED on the Day 1 command (-s only): four weeks later the same seed gave 1,151 patients, not 1,142. -s pins the patient RNG but the clinician seed (-cs), reference date (-r) and end date (-e) all default to the wall clock. Each was found by fixing one and seeing what still moved. With all four, two runs are identical in content. Data regenerated 2026-09-20; every number here is from the pinned output. See DAY_1_DECISIONS.md D2.</t>
         </is>
       </c>
     </row>
@@ -4073,7 +4077,7 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>Decided Day 1 — the evidence arrived early. Anchoring on 44054006 alone misses 72 patients who carry a diabetic complication with no underlying dx code (45% of cohort, and the sickest half). Prediabetes 714628002 excluded: 430 patients, would triple the denominator. 0 of 819 diabetes rows have a stop date, so "ever recorded" needs no date logic. See pipeline/cohort.py.</t>
+          <t>Decided Day 1 — the evidence arrived early. Anchoring on 44054006 alone misses 73 patients who carry a diabetic complication with no underlying dx code (45% of cohort, and the sickest half). Prediabetes 714628002 excluded: 439 patients, would triple the denominator. 0 of 835 diabetes rows have a stop date, so "ever recorded" needs no date logic. See pipeline/cohort.py.</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4297,7 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Glucose is the larger table (9,879 vs 8,749) and covers more of the cohort. Both are reasons to reject it.</t>
+          <t>Glucose is the larger table (10,439 vs 8,941) and covers more of the cohort. Both are reasons to reject it.</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -4313,7 +4317,7 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>A1c integrates ~3 months of blood sugar; glucose is a snapshot. In our own data the within-patient, within-year spread is 6.2% of the mean for A1c vs 21.0% for glucose. Glucose is also drawn on everyone incidentally — 160 of 161 cohort patients have one vs 131 with an A1c — so its absence carries no signal. And HEDIS specifies A1c; no measure anywhere requires an annual glucose.</t>
+          <t>A1c integrates ~3 months of blood sugar; glucose is a snapshot. In our own data the within-patient, within-year spread is 6.7% of the mean for A1c vs 21.3% for glucose. Glucose is also drawn on everyone incidentally — 159 of 161 cohort patients have one vs 133 with an A1c — so its absence carries no signal. And HEDIS specifies A1c; no measure anywhere requires an annual glucose.</t>
         </is>
       </c>
     </row>
@@ -4372,7 +4376,7 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>claims_transactions alone is 1,031,224 rows — 40% of total volume with no clinical role.</t>
+          <t>claims_transactions alone is 1,094,500 rows — 40% of total volume with no clinical role.</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
@@ -4856,7 +4860,7 @@
         </is>
       </c>
       <c r="C5" s="12" t="n">
-        <v>1142</v>
+        <v>1153</v>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
@@ -4879,7 +4883,7 @@
         </is>
       </c>
       <c r="C6" s="12" t="n">
-        <v>65350</v>
+        <v>67755</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -4902,7 +4906,7 @@
         </is>
       </c>
       <c r="C7" s="12" t="n">
-        <v>40105</v>
+        <v>40811</v>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
@@ -4925,7 +4929,7 @@
         </is>
       </c>
       <c r="C8" s="12" t="n">
-        <v>836111</v>
+        <v>870510</v>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
@@ -4948,7 +4952,7 @@
         </is>
       </c>
       <c r="C9" s="12" t="n">
-        <v>56228</v>
+        <v>59273</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
@@ -5022,7 +5026,7 @@
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>2.3 / 5.2 / 8.8  (n=8,749; 993 below DQ3 floor of 3.0 → revise floor to 2.0)</t>
+          <t>2.3 / 4.1 / 8.8  (n=8,941; 951 below DQ3 floor of 3.0 → revise floor to 2.0)</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
@@ -5047,7 +5051,7 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>0.0%  (0 of 819 diabetes condition rows have a STOP date)</t>
+          <t>0.0%  (0 of 835 diabetes condition rows have a STOP date)</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
@@ -5262,7 +5266,7 @@
         </is>
       </c>
       <c r="C23" s="12" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Day 2: corrupt.py injects six defect classes and logs ground truth
249 rows damaged across Bronze, none carrying more than one defect:
D1 40 duplicate encounters, D2 150 orphan observations, D3 20 A1c
values of 250 (sampled from cohort patients so D4 moves the gap count),
D4 8 future birth dates, D5 25 swapped admission/discharge, D6 6
duplicate patient registrations under a derived Id.

Idempotent by reloading Bronze first; sampling is ORDER BY md5(key) so
the log is byte-identical across runs (V2.3, V2.4). Every entry resolves
to exactly the expected row (V2.1). Cohort still 161 (V2.7).

Workbook: D3 volumes, DQ Matrix rows injected, Learning Log #2 and #13.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build-plan/Clinical_Care_Gap_Build_Plan.xlsx
+++ b/build-plan/Clinical_Care_Gap_Build_Plan.xlsx
@@ -1796,7 +1796,7 @@
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr"/>
@@ -1832,10 +1832,14 @@
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H19" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>D3 recorded: 40/150/20/8/25/6 = 249 rows, all under 1% of table.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="62" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -1868,7 +1872,7 @@
       </c>
       <c r="G20" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H20" s="13" t="inlineStr"/>
@@ -1904,7 +1908,7 @@
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H21" s="13" t="inlineStr"/>
@@ -1940,7 +1944,7 @@
       </c>
       <c r="G22" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr"/>
@@ -1976,7 +1980,7 @@
       </c>
       <c r="G23" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H23" s="13" t="inlineStr"/>
@@ -2012,7 +2016,7 @@
       </c>
       <c r="G24" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H24" s="13" t="inlineStr"/>
@@ -2048,7 +2052,7 @@
       </c>
       <c r="G25" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H25" s="13" t="inlineStr"/>
@@ -2084,10 +2088,14 @@
       </c>
       <c r="G26" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H26" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H26" s="13" t="inlineStr">
+        <is>
+          <t>data/injected_defects.json - 249 entries, no timestamps so V2.3 can diff it. Committed.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="62" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
@@ -2120,10 +2128,14 @@
       </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H27" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="inlineStr">
+        <is>
+          <t>Reload-first: corrupt.py calls load_bronze before injecting. V2.3 + V2.4 pass; JSON byte-identical across runs.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="62" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -4012,8 +4024,16 @@
           <t>Day 2</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr"/>
-      <c r="G7" s="13" t="inlineStr"/>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>D1 40 · D2 150 · D3 20 · D4 8 · D5 25 · D6 6  (≈249 rows)</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>Nothing exceeds 1% of its table (largest is D4 at 0.7% of patients). Enough that quarantine reads as a real work queue on P2, small enough that the 161-patient cohort and its 133 A1c-tested patients survive (V2.7). D3 rows are sampled from cohort patients so Decision D4 (remediate vs quarantine) visibly moves the gap count on Day 4.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="74" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -4511,7 +4531,9 @@
           <t>DQ1 — encounter uniqueness</t>
         </is>
       </c>
-      <c r="F5" s="12" t="n"/>
+      <c r="F5" s="12" t="n">
+        <v>40</v>
+      </c>
       <c r="G5" s="12" t="n"/>
       <c r="H5" s="8">
         <f>IF(COUNT(G5)=0,"",IF(G5&gt;0,"YES","NO"))</f>
@@ -4545,7 +4567,9 @@
           <t>DQ2 — referential integrity</t>
         </is>
       </c>
-      <c r="F6" s="12" t="n"/>
+      <c r="F6" s="12" t="n">
+        <v>150</v>
+      </c>
       <c r="G6" s="12" t="n"/>
       <c r="H6" s="8">
         <f>IF(COUNT(G6)=0,"",IF(G6&gt;0,"YES","NO"))</f>
@@ -4579,7 +4603,9 @@
           <t>DQ3 — A1c plausibility</t>
         </is>
       </c>
-      <c r="F7" s="12" t="n"/>
+      <c r="F7" s="12" t="n">
+        <v>20</v>
+      </c>
       <c r="G7" s="12" t="n"/>
       <c r="H7" s="8">
         <f>IF(COUNT(G7)=0,"",IF(G7&gt;0,"YES","NO"))</f>
@@ -4613,7 +4639,9 @@
           <t>DQ4 — birth date sanity</t>
         </is>
       </c>
-      <c r="F8" s="12" t="n"/>
+      <c r="F8" s="12" t="n">
+        <v>8</v>
+      </c>
       <c r="G8" s="12" t="n"/>
       <c r="H8" s="8">
         <f>IF(COUNT(G8)=0,"",IF(G8&gt;0,"YES","NO"))</f>
@@ -4647,7 +4675,9 @@
           <t>DQ5 — encounter chronology</t>
         </is>
       </c>
-      <c r="F9" s="12" t="n"/>
+      <c r="F9" s="12" t="n">
+        <v>25</v>
+      </c>
       <c r="G9" s="12" t="n"/>
       <c r="H9" s="8">
         <f>IF(COUNT(G9)=0,"",IF(G9&gt;0,"YES","NO"))</f>
@@ -4681,7 +4711,9 @@
           <t>DQ6 — patient identity</t>
         </is>
       </c>
-      <c r="F10" s="12" t="n"/>
+      <c r="F10" s="12" t="n">
+        <v>6</v>
+      </c>
       <c r="G10" s="12" t="n"/>
       <c r="H10" s="8">
         <f>IF(COUNT(G10)=0,"",IF(G10&gt;0,"YES","NO"))</f>
@@ -5074,7 +5106,9 @@
           <t>Rows corrupted (total)</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr"/>
+      <c r="C14" s="12" t="n">
+        <v>249</v>
+      </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
           <t>P2 pipeline page</t>
@@ -5414,7 +5448,11 @@
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr"/>
-      <c r="F6" s="13" t="inlineStr"/>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Nothing about real-world performance: Synthea has no typos, no interface replays, no duplicate registrations, and names carry numeric suffixes so identity matching is trivially clean. The defects are the ones I injected, so catch rate measures my checks against my own defect list, not against reality. Also learned: synthetic does not mean deterministic - the generator has a 'now' that follows the wall clock unless pinned (see #13).</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="10" t="n">
@@ -5656,7 +5694,11 @@
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr"/>
-      <c r="F17" s="13" t="inlineStr"/>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Only if every source of randomness AND every source of time is pinned. I tested it: -s alone failed four weeks later (1,151 patients, not 1,142) because Synthea's clinician seed, reference date and end date all default to the wall clock. Now -s -cs -r -e are all fixed and two runs match in content. 'Reproducible' means same content, not same bytes - the export is multi-threaded so row order varies; verify with a sorted diff or DuckDB EXCEPT, never md5. The README numbers are guaranteed by the pinned command in D2 plus the Bronze row-count check, not by a claim.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="10" t="n">

</xml_diff>

<commit_message>
Day 7: clean-clone fixes found by V7.11
Cloning the repo and following the README exactly surfaced two things a
reviewer would hit. run_all.py --generate now downloads the Synthea jar
itself (with -L, and a clear message when java is missing), and running
without --generate on a fresh clone prints a sentence explaining what to
run instead of a DuckDB IOException. The README documents the Java 17
requirement and the web app's own install step.

D12 recorded: P4 ships no model. A static site has nowhere to hold an API
key, and the cut buys something a hosted model would not - the SQL shown
is the SQL executed.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build-plan/Clinical_Care_Gap_Build_Plan.xlsx
+++ b/build-plan/Clinical_Care_Gap_Build_Plan.xlsx
@@ -3516,7 +3516,7 @@
       </c>
       <c r="G64" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr"/>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="G65" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H65" s="13" t="inlineStr"/>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="G66" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr"/>
@@ -3624,10 +3624,14 @@
       </c>
       <c r="G67" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H67" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H67" s="13" t="inlineStr">
+        <is>
+          <t>Allowlist on the statement's actual verb. A test found WITH x AS (SELECT 1) DELETE FROM patients passing - now walks the CTE list. 19/19 cases.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="62" customHeight="1">
       <c r="A68" s="8" t="inlineStr">
@@ -3660,10 +3664,14 @@
       </c>
       <c r="G68" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H68" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H68" s="13" t="inlineStr">
+        <is>
+          <t>Free-text refuses anything unmatched with one sentence naming what it can answer.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="62" customHeight="1">
       <c r="A69" s="8" t="inlineStr">
@@ -3696,10 +3704,14 @@
       </c>
       <c r="G69" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H69" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H69" s="13" t="inlineStr">
+        <is>
+          <t>Audit log on P4: role, question, SQL, rows, outcome. Refusals logged too.</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="62" customHeight="1">
       <c r="A70" s="8" t="inlineStr">
@@ -3732,7 +3744,7 @@
       </c>
       <c r="G70" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H70" s="13" t="inlineStr"/>
@@ -3768,7 +3780,7 @@
       </c>
       <c r="G71" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H71" s="13" t="inlineStr"/>
@@ -3804,10 +3816,14 @@
       </c>
       <c r="G72" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H72" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H72" s="13" t="inlineStr">
+        <is>
+          <t>Written from this week's real friction: DuckDB single-writer, the four-flag reproducibility failure, quarantine as a dead-letter queue.</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="62" customHeight="1">
       <c r="A73" s="8" t="inlineStr">
@@ -4393,8 +4409,16 @@
           <t>Day 7</t>
         </is>
       </c>
-      <c r="F16" s="13" t="inlineStr"/>
-      <c r="G16" s="13" t="inlineStr"/>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>No model. Ten preset questions with hand-written SQL, run in DuckDB-WASM in the browser.</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>D9 made the site a static export, so there is nowhere to hold an API key - a key shipped to the browser is a public key. The plan allows this cut ('ten working chips and no free-text box still demonstrates the idea') and it buys something a hosted model would not: the SQL displayed is literally the SQL executed, against the same Parquet the site ships, so a reviewer can copy it and get the same rows. The free-text box matches wording to the presets and refuses everything else by naming what it can answer. The page says it is a query builder, not a language model.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="74" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
@@ -5470,7 +5494,7 @@
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>12 s from a deleted warehouse to Gold (run_all.py --fresh); +4 min with --generate</t>
+          <t>13 s warehouse-to-Gold; ~4 min with --generate (Synthea + jar download)</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Add REMAINING.md; correct stale tracker statuses and record D8, D9
The tracker still showed Day 5 and tasks 1.12-1.13 as not started when
they shipped days ago, and D9 was decided on Day 5 but only ever written
into a commit message. Both corrected, so the audit reflects reality.

D8 recorded as a no: quarantine stays a dead-letter queue in v1, because
a half-built replay path would make the reconciliation assertion
ambiguous, and that is the one guarantee worth keeping exact.

REMAINING.md covers the four things that need a person rather than code:
the role matrix, the Learning Log, the Loom (with a timed shot list) and
the three-minute test.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build-plan/Clinical_Care_Gap_Build_Plan.xlsx
+++ b/build-plan/Clinical_Care_Gap_Build_Plan.xlsx
@@ -1724,10 +1724,14 @@
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H16" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>load_bronze.py, all_varchar=true, verified V1.5/V1.6/V1.7 on every run.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="62" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
@@ -1760,7 +1764,7 @@
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H17" s="13" t="inlineStr"/>
@@ -2888,7 +2892,7 @@
       </c>
       <c r="G47" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H47" s="13" t="inlineStr"/>
@@ -2924,10 +2928,14 @@
       </c>
       <c r="G48" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H48" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H48" s="13" t="inlineStr">
+        <is>
+          <t>D9: static export. JSON for the pages, Parquet for DuckDB-WASM on P4.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="62" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
@@ -2960,7 +2968,7 @@
       </c>
       <c r="G49" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H49" s="13" t="inlineStr"/>
@@ -2996,7 +3004,7 @@
       </c>
       <c r="G50" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -3032,7 +3040,7 @@
       </c>
       <c r="G51" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H51" s="13" t="inlineStr"/>
@@ -3068,7 +3076,7 @@
       </c>
       <c r="G52" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr"/>
@@ -3104,7 +3112,7 @@
       </c>
       <c r="G53" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H53" s="13" t="inlineStr"/>
@@ -3140,7 +3148,7 @@
       </c>
       <c r="G54" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr"/>
@@ -3176,7 +3184,7 @@
       </c>
       <c r="G55" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H55" s="13" t="inlineStr"/>
@@ -3212,10 +3220,14 @@
       </c>
       <c r="G56" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H56" s="13" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H56" s="13" t="inlineStr">
+        <is>
+          <t>GitHub Pages (Vercel needs an interactive login). Live since Day 5.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="62" customHeight="1">
       <c r="A57" s="8" t="inlineStr">
@@ -4277,8 +4289,16 @@
           <t>Day 4</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr"/>
-      <c r="G12" s="13" t="inlineStr"/>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>No. Quarantine is a dead-letter queue in v1; the replay path is named as scale work.</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>Reprocessing needs three things this project does not have: a replay path, a resolved_at column, and a rule for whether a replayed row enters Silver under its original load date or today's. Building a half version would make the reconciliation assertion ambiguous, which is the one guarantee worth keeping exact. Written up in DATA_QUALITY_SPEC.md under what I would do differently at scale.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="74" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
@@ -4306,8 +4326,16 @@
           <t>Day 5</t>
         </is>
       </c>
-      <c r="F13" s="13" t="inlineStr"/>
-      <c r="G13" s="13" t="inlineStr"/>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Static export at build time. JSON for the pages, Parquet for DuckDB-WASM.</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>Decided Day 5, recorded here late. A server runtime holding clinical.duckdb would have failed on a serverless filesystem, and the deploy had to work on Day 5 rather than Day 7. Exporting both formats costs 458 KB: the pages render from JSON with no engine to load, and P4 queries the Parquet in the browser so the SQL it shows is the SQL that ran. The trade-off accepted is that the site reads a snapshot - re-running the pipeline without re-exporting leaves it stale, which is why export_web is the last stage of run_all.py.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="74" customHeight="1">
       <c r="A14" s="8" t="inlineStr">

</xml_diff>